<commit_message>
big change going to happen, this is not an auto save but need to save
</commit_message>
<xml_diff>
--- a/ref/task_margin.xlsx
+++ b/ref/task_margin.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mongk\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mongk\Desktop\milestone\ref\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9C649F81-8BA8-432E-9AF6-6314793107E8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8214616B-380D-4284-9633-C9059737AB82}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="27096" windowHeight="16296" xr2:uid="{3C2C6E59-DEC1-41FA-96DF-BFFAAA78D3A5}"/>
   </bookViews>
@@ -1177,7 +1177,7 @@
         <v>6</v>
       </c>
       <c r="B5">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="C5">
         <v>1</v>
@@ -1187,7 +1187,7 @@
       </c>
       <c r="G5">
         <f t="shared" si="0"/>
-        <v>35</v>
+        <v>30</v>
       </c>
       <c r="I5">
         <v>25</v>
@@ -1207,7 +1207,7 @@
         <v>7</v>
       </c>
       <c r="B6">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="C6">
         <v>1</v>
@@ -1217,7 +1217,7 @@
       </c>
       <c r="G6">
         <f t="shared" si="0"/>
-        <v>35</v>
+        <v>30</v>
       </c>
       <c r="I6">
         <v>30</v>
@@ -1237,10 +1237,10 @@
         <v>8</v>
       </c>
       <c r="B7">
-        <v>5</v>
+        <v>25</v>
       </c>
       <c r="C7">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E7" s="2">
         <v>1</v>
@@ -1267,17 +1267,17 @@
         <v>9</v>
       </c>
       <c r="B8">
-        <v>5</v>
+        <v>20</v>
       </c>
       <c r="C8">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E8" s="2">
         <v>1</v>
       </c>
       <c r="G8">
         <f t="shared" si="0"/>
-        <v>45</v>
+        <v>40</v>
       </c>
       <c r="L8">
         <v>28</v>
@@ -1291,15 +1291,17 @@
         <v>51</v>
       </c>
       <c r="B9">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="C9">
         <v>1</v>
       </c>
-      <c r="E9" s="2"/>
+      <c r="E9" s="2">
+        <v>1</v>
+      </c>
       <c r="G9">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>25</v>
       </c>
       <c r="L9">
         <v>29</v>
@@ -1313,15 +1315,17 @@
         <v>52</v>
       </c>
       <c r="B10">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="C10">
         <v>1</v>
       </c>
-      <c r="E10" s="2"/>
+      <c r="E10" s="2">
+        <v>1</v>
+      </c>
       <c r="G10">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>35</v>
       </c>
       <c r="L10">
         <v>31</v>
@@ -1335,15 +1339,17 @@
         <v>53</v>
       </c>
       <c r="B11">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="C11">
         <v>1</v>
       </c>
-      <c r="E11" s="2"/>
+      <c r="E11" s="2">
+        <v>1</v>
+      </c>
       <c r="G11">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>30</v>
       </c>
       <c r="L11">
         <v>33</v>
@@ -1357,15 +1363,17 @@
         <v>54</v>
       </c>
       <c r="B12">
-        <v>5</v>
+        <v>25</v>
       </c>
       <c r="C12">
-        <v>2</v>
-      </c>
-      <c r="E12" s="2"/>
+        <v>1</v>
+      </c>
+      <c r="E12" s="2">
+        <v>1</v>
+      </c>
       <c r="G12">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>45</v>
       </c>
     </row>
     <row r="13" spans="1:13" x14ac:dyDescent="0.3">
@@ -1373,15 +1381,17 @@
         <v>10</v>
       </c>
       <c r="B13">
-        <v>15</v>
+        <v>35</v>
       </c>
       <c r="C13">
-        <v>2</v>
-      </c>
-      <c r="E13" s="2"/>
+        <v>1</v>
+      </c>
+      <c r="E13" s="2">
+        <v>1</v>
+      </c>
       <c r="G13">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>55</v>
       </c>
     </row>
     <row r="14" spans="1:13" x14ac:dyDescent="0.3">
@@ -1389,15 +1399,17 @@
         <v>11</v>
       </c>
       <c r="B14">
-        <v>15</v>
+        <v>35</v>
       </c>
       <c r="C14">
-        <v>2</v>
-      </c>
-      <c r="E14" s="2"/>
+        <v>1</v>
+      </c>
+      <c r="E14" s="2">
+        <v>1</v>
+      </c>
       <c r="G14">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>55</v>
       </c>
     </row>
     <row r="15" spans="1:13" x14ac:dyDescent="0.3">
@@ -1405,10 +1417,10 @@
         <v>12</v>
       </c>
       <c r="B15">
-        <v>5</v>
+        <v>25</v>
       </c>
       <c r="C15">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E15" s="2">
         <v>1</v>
@@ -1423,10 +1435,10 @@
         <v>13</v>
       </c>
       <c r="B16">
-        <v>15</v>
+        <v>35</v>
       </c>
       <c r="C16">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E16" s="2">
         <v>1</v>
@@ -1441,17 +1453,17 @@
         <v>14</v>
       </c>
       <c r="B17">
-        <v>5</v>
+        <v>30</v>
       </c>
       <c r="C17">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E17" s="2">
         <v>1</v>
       </c>
       <c r="G17">
         <f t="shared" si="0"/>
-        <v>25</v>
+        <v>30</v>
       </c>
     </row>
     <row r="18" spans="1:12" x14ac:dyDescent="0.3">
@@ -1615,17 +1627,17 @@
         <v>21</v>
       </c>
       <c r="B24">
+        <v>35</v>
+      </c>
+      <c r="C24">
         <v>0</v>
       </c>
-      <c r="C24">
-        <v>2</v>
-      </c>
       <c r="E24" s="2">
         <v>1</v>
       </c>
       <c r="G24">
         <f t="shared" si="0"/>
-        <v>40</v>
+        <v>35</v>
       </c>
     </row>
     <row r="25" spans="1:12" x14ac:dyDescent="0.3">
@@ -1633,17 +1645,17 @@
         <v>22</v>
       </c>
       <c r="B25">
-        <v>5</v>
+        <v>30</v>
       </c>
       <c r="C25">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E25" s="2">
         <v>1</v>
       </c>
       <c r="G25">
         <f t="shared" si="0"/>
-        <v>25</v>
+        <v>30</v>
       </c>
       <c r="I25" s="1" t="s">
         <v>44</v>
@@ -1662,7 +1674,7 @@
       </c>
       <c r="H27">
         <f>SUM(G:G)/20</f>
-        <v>20.5</v>
+        <v>32.25</v>
       </c>
       <c r="I27" s="4" t="s">
         <v>47</v>
@@ -1676,7 +1688,7 @@
       </c>
       <c r="L27" s="3">
         <f>H27+J27</f>
-        <v>23.3</v>
+        <v>35.049999999999997</v>
       </c>
     </row>
     <row r="28" spans="1:12" x14ac:dyDescent="0.3">

</xml_diff>